<commit_message>
error el guardar bio
ERROR AL GUARDAR BIOMETRICO

descarga de archivo

actualizacion

error query

Error en query de falta por omision

configuracion biometrico

activo modificaiocn de datos biometricos

orden plaza

Envia el ultimo numero de plaza en la busqueda

cambios general empelados

Empleados

asistencia

tabla

asistencias

Movimientos

correcion movimeintos

querys asistencia

a

boton

boton eliminar faltas y retardos

null

no tomar en cuanta no dispositivo null

query faltas

a

archivojustificacion-mm-dd

Actualizacion de fomato de aaaa

MENU_DESPLEGABLE

MOVIMIENTOS

sin cambio

Update MovimientosM.php

orden movimeinto

excluidos

Excluidos de checada controlador y view

orden de no_plaza

avance pagina

avance pagina emplados

movimento y plazas

Cambios en views nueva base movimientos y plazas

faltas asistencia

cambvio

faltas

Código certificación

SE elimina de formulario

DetallePLazas

Detalle PLazas if
</commit_message>
<xml_diff>
--- a/assets/Formato/LAYOUT_JUSTIFICACION.xlsx
+++ b/assets/Formato/LAYOUT_JUSTIFICACION.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\sirh\assets\Formato\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joaquin.hernandez\Desktop\REGISTROS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E17CB908-ED81-4B9F-89AC-59916EC3EC21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A57CFEC0-EFD8-4153-B452-C46168980BDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CDFFC4D4-785C-409B-827D-72446BEA2B34}"/>
   </bookViews>
@@ -41,9 +41,6 @@
     <t>RFC*</t>
   </si>
   <si>
-    <t>FECHA (YYYY/MM/DD) *</t>
-  </si>
-  <si>
     <t>OBSERVACIONES</t>
   </si>
   <si>
@@ -51,6 +48,9 @@
   </si>
   <si>
     <t>TIPO DE FALTA/RETARDO</t>
+  </si>
+  <si>
+    <t>FECHA (YYYY-MM-DD) *</t>
   </si>
 </sst>
 </file>
@@ -467,16 +467,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>